<commit_message>
Remove comma from label to simplify CSV parsing
</commit_message>
<xml_diff>
--- a/data_raw/OS-Inventory-list-20260202.xlsx
+++ b/data_raw/OS-Inventory-list-20260202.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xiuqili-local/Documents/GitHub/UCSB-Library-OSSSI/data_raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gjanee-local/work/UCSB-Library-OSSSI/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2DD706F-B2C0-D444-91FB-B4DAAD92DB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFDB9023-E5C9-DC45-97A9-0A91D637B691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6740" yWindow="1020" windowWidth="30240" windowHeight="18880" xr2:uid="{1509BDA8-4FD2-7641-BB7D-D0BB426F409D}"/>
+    <workbookView xWindow="2940" yWindow="1020" windowWidth="30240" windowHeight="18880" xr2:uid="{1509BDA8-4FD2-7641-BB7D-D0BB426F409D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -268,9 +268,6 @@
     <t>Education</t>
   </si>
   <si>
-    <t>LibGuides, OS-themed</t>
-  </si>
-  <si>
     <t>Data Access Education</t>
   </si>
   <si>
@@ -335,6 +332,9 @@
   </si>
   <si>
     <t>R&amp;E SRC</t>
+  </si>
+  <si>
+    <t>LibGuides (OS-themed)</t>
   </si>
 </sst>
 </file>
@@ -946,7 +946,7 @@
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -980,7 +980,7 @@
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -1022,7 +1022,7 @@
         <v>31</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C15" s="4">
         <v>14</v>
@@ -1069,7 +1069,7 @@
         <v>20</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>52</v>
@@ -1132,7 +1132,7 @@
         <v>18</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>8</v>
@@ -1153,7 +1153,7 @@
         <v>20</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>8</v>
@@ -1174,7 +1174,7 @@
         <v>20</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>8</v>
@@ -1195,7 +1195,7 @@
         <v>20</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>32</v>
@@ -1216,7 +1216,7 @@
         <v>20</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>8</v>
@@ -1228,7 +1228,7 @@
         <v>35</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="C25" s="8">
         <v>24</v>
@@ -1237,10 +1237,10 @@
         <v>20</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G25" s="7"/>
     </row>
@@ -1279,7 +1279,7 @@
         <v>20</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>7</v>
@@ -1291,7 +1291,7 @@
         <v>35</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C28" s="8">
         <v>27</v>
@@ -1321,7 +1321,7 @@
         <v>20</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>8</v>
@@ -1432,7 +1432,7 @@
         <v>8</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1475,10 +1475,10 @@
         <v>49</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1616,7 +1616,7 @@
         <v>8</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1633,13 +1633,13 @@
         <v>20</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F43" s="5" t="s">
         <v>7</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1662,7 +1662,7 @@
         <v>32</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1682,10 +1682,10 @@
         <v>22</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1725,7 +1725,7 @@
         <v>20</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>8</v>
@@ -1746,7 +1746,7 @@
         <v>20</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>7</v>
@@ -1770,7 +1770,7 @@
         <v>21</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G49" s="9"/>
     </row>
@@ -1811,7 +1811,7 @@
         <v>18</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>8</v>
@@ -1856,7 +1856,7 @@
         <v>76</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G53" s="9"/>
     </row>

</xml_diff>